<commit_message>
Add vendor pass module
</commit_message>
<xml_diff>
--- a/public/files/VendorTemplateNew.xlsx
+++ b/public/files/VendorTemplateNew.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="18.71" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,8 @@
     <col width="18.71" bestFit="1" customWidth="1" min="31" max="31"/>
     <col width="13.997" bestFit="1" customWidth="1" min="32" max="32"/>
     <col width="43.561" bestFit="1" customWidth="1" min="33" max="33"/>
+    <col width="16" customWidth="1" min="34" max="34"/>
+    <col width="16" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -646,6 +648,16 @@
           <t>Remark</t>
         </is>
       </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>License Class</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>License Expiry</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -803,11 +815,21 @@
           <t>Sample row — delete before uploading</t>
         </is>
       </c>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>B,D</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Fields marked * are required. Leave App No blank to auto-generate. Resident must be Malaysian or Non-Malaysian. Worker Type must be Permanent or Temporary. In/Out Bound must be INSIDE or OUTSIDE. Type Of Registration must be TENANT or NON-TENANT. Payment must be NONE, ONLINE or CASH. Sex must be Male or Female. IC No. / Passport accepts a 12-digit IC number (no dashes) or a passport number. Location Access accepts one or more of: annexe_building, kpk_gate, ksb_phase2_gate, phase1 (comma-separated, no spaces). Dates (Date Of Birth, Pass Expiry): DD/MM/YYYY.</t>
+          <t>Fields marked * are required. Leave App No blank to auto-generate. Resident must be Malaysian or Non-Malaysian. Worker Type must be Permanent or Temporary. In/Out Bound must be INSIDE or OUTSIDE. Type Of Registration must be TENANT or NON-TENANT. Payment must be NONE, ONLINE or CASH. Sex must be Male or Female. IC No. / Passport accepts a 12-digit IC number (no dashes) or a passport number. Location Access accepts one or more of the active location codes set up under Vendor &gt; Locations (comma-separated, no spaces). Dates (Date Of Birth, Pass Expiry): DD/MM/YYYY. License Class and License Expiry are optional — License Class accepts one letter (e.g. B) or several comma-separated (e.g. B,C,D); License Expiry uses DD/MM/YYYY.</t>
         </is>
       </c>
     </row>

</xml_diff>